<commit_message>
auto-publish commission xlsx: client-summary upload 2026-01-01
</commit_message>
<xml_diff>
--- a/commission/karin/2026-05.xlsx
+++ b/commission/karin/2026-05.xlsx
@@ -675,7 +675,7 @@
         <v>1</v>
       </c>
       <c r="H1" s="3">
-        <v>3878.59</v>
+        <v>3935</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1205,10 +1205,10 @@
         <v>37</v>
       </c>
       <c r="F38" s="10">
-        <v>2435.88</v>
+        <v>3000</v>
       </c>
       <c r="H38" s="11">
-        <v>243.58800000000002</v>
+        <v>300</v>
       </c>
     </row>
     <row r="39" spans="2:8" x14ac:dyDescent="0.25">
@@ -1282,13 +1282,13 @@
         <v>39</v>
       </c>
       <c r="F42" s="13">
-        <v>1835.88</v>
+        <v>2400</v>
       </c>
       <c r="G42" s="16">
         <v>0.1</v>
       </c>
       <c r="H42" s="17">
-        <v>183.58800000000002</v>
+        <v>240</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -1631,10 +1631,10 @@
         <v>52</v>
       </c>
       <c r="F69" s="19">
-        <v>38785.88</v>
+        <v>39350</v>
       </c>
       <c r="H69" s="20">
-        <v>3878.59</v>
+        <v>3935</v>
       </c>
     </row>
   </sheetData>

</xml_diff>